<commit_message>
Added Date variable and import excel export
</commit_message>
<xml_diff>
--- a/backend/receipts_export.xlsx
+++ b/backend/receipts_export.xlsx
@@ -425,38 +425,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>receipt_id</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>vendor_name</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>image_path</t>
+          <t>Vendor</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Amount</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>user_id</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>Date</t>
         </is>
       </c>
     </row>
@@ -466,26 +466,50 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>S_4545</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>WALMAR &gt;&lt;.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>uploads\receipt-ocr-original.webp</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>93.62</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>S_4545</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>93.62</v>
+      <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>S_0001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BER GHOTEL</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>